<commit_message>
chore(preview): NVDA outputs regeneres
</commit_message>
<xml_diff>
--- a/preview/NVDA/NVDA_financials.xlsx
+++ b/preview/NVDA/NVDA_financials.xlsx
@@ -13932,7 +13932,7 @@
         <v>226</v>
       </c>
       <c r="H95" s="233" t="n">
-        <v>194.24</v>
+        <v>194.51</v>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
@@ -14064,7 +14064,7 @@
       <c r="F100" s="426" t="n"/>
       <c r="G100" s="426" t="n"/>
       <c r="H100" s="427" t="n">
-        <v>0.0427</v>
+        <v>0.0428</v>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
@@ -20030,7 +20030,7 @@
         </is>
       </c>
       <c r="C14" s="642" t="n">
-        <v>194.29</v>
+        <v>194.51</v>
       </c>
     </row>
     <row r="15">
@@ -34085,7 +34085,7 @@
         </is>
       </c>
       <c r="D9" s="588" t="n">
-        <v>252.4</v>
+        <v>252.35</v>
       </c>
       <c r="E9" s="589" t="n">
         <v>395888.3</v>
@@ -34125,7 +34125,7 @@
         </is>
       </c>
       <c r="D10" s="588" t="n">
-        <v>62.62</v>
+        <v>62.53</v>
       </c>
       <c r="E10" s="589" t="n">
         <v>347346.11</v>
@@ -34165,7 +34165,7 @@
         </is>
       </c>
       <c r="D11" s="588" t="n">
-        <v>131.76</v>
+        <v>131.6</v>
       </c>
       <c r="E11" s="589" t="n">
         <v>143028.08</v>
@@ -34245,7 +34245,7 @@
         </is>
       </c>
       <c r="D13" s="591" t="n">
-        <v>379.33</v>
+        <v>379.31</v>
       </c>
       <c r="E13" s="592" t="n">
         <v>7625004.02</v>

</xml_diff>